<commit_message>
12 yeni karakter: Hiyori, Lilynette, Harribel'in Fracción'ı ve diğerleri
Hiyori Sarugaki, Lilynette Gingerbuck, Emilou Apacci, Franceska Mila Rose,
Cyan Sung-Sun, Grand Fisher, Ggio Vega, Akon, Kiyone Kotetsu,
Sentarō Kotsubaki, Moe Shishigawara, Royd Lloyd. Classic 113 -> 125,
Splash 108 -> 120, Bankai 55 -> 60.

Saç/yaş/konum override'ları wiki Appearance metni ve görsellerle girildi.
Akon ve Hiyori 110 yıl önce sahnede: 101-1000.

- build_bankai: havuzda zaten olan salım adı ikinci karaktere eklenmez
  (Lilynette'in Los Lobos'u Starrk'ınki; iki doğru cevap olurdu).
- scrape_splash: CamelCase bölme aksanlardan önce yapılıyordu,
  "SuìFēng" bölünmeyip Suì-Fēng'li bir kare Ggio'ya seçiliyordu.
  Var olan görseli kayıtlı yoldan kontrol ediyor (görünen ad değişince
  yeniden indirmesin). Ggio, Lilynette, Akon, Moe, Royd görselleri
  elle seçildi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bleachdle-ses.xlsx
+++ b/bleachdle-ses.xlsx
@@ -655,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -759,7 +759,11 @@
           <t>Byakuya_Kuchiki</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
@@ -796,7 +800,11 @@
           <t>Chōjirō_Sasakibe</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr"/>
@@ -833,7 +841,11 @@
           <t>Genryūsai_Shigekuni_Yamamoto</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
@@ -870,7 +882,11 @@
           <t>Gin_Ichimaru</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
@@ -907,7 +923,11 @@
           <t>Ichigo_Kurosaki</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
@@ -944,7 +964,11 @@
           <t>Ikkaku_Madarame</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
@@ -981,7 +1005,11 @@
           <t>Kaname_Tōsen</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
@@ -1018,7 +1046,11 @@
           <t>Kensei_Muguruma</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
@@ -1055,7 +1087,11 @@
           <t>Kisuke_Urahara</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
@@ -1092,7 +1128,11 @@
           <t>Mayuri_Kurotsuchi</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
@@ -1129,7 +1169,11 @@
           <t>Renji_Abarai</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
@@ -1166,7 +1210,11 @@
           <t>Retsu_Unohana</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
@@ -1203,7 +1251,11 @@
           <t>Rukia_Kuchiki</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
@@ -1240,7 +1292,11 @@
           <t>Rōjūrō_Ōtoribashi</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -1277,7 +1333,11 @@
           <t>Sajin_Komamura</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
@@ -1314,7 +1374,11 @@
           <t>Senjumaru_Shutara</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
@@ -1351,7 +1415,11 @@
           <t>Shinji_Hirako</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
@@ -1388,7 +1456,11 @@
           <t>Shunsui_Kyōraku</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
@@ -1425,7 +1497,11 @@
           <t>Sui_Feng</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -1462,7 +1538,11 @@
           <t>Tōshirō_Hitsugaya</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
@@ -1499,7 +1579,11 @@
           <t>Aaroniero_Arruruerie</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1536,7 +1620,11 @@
           <t>Baraggan_Louisenbairn</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
@@ -1573,7 +1661,11 @@
           <t>Cirucci_Sanderwicci</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
@@ -1610,7 +1702,11 @@
           <t>Coyote_Starrk</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
@@ -1619,17 +1715,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Dordoni_Alessandro_Del_Socaccio</t>
+          <t>Cyan_Sung_Sun</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Dordoni Alessandro Del Socaccio</t>
+          <t>Cyan Sung-Sun</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Giralda</t>
+          <t>Anaconda</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1639,12 +1735,12 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Giralda" çağrısı</t>
+          <t>"Resurrección: Anaconda" çağrısı</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Dordoni_Alessandro_Del_Socaccio</t>
+          <t>Cyan_Sung_Sun</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1656,17 +1752,17 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Findorr_Calius</t>
+          <t>Dordoni_Alessandro_Del_Socaccio</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Findorr Calius</t>
+          <t>Dordoni Alessandro Del Socaccio</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Pinza Aguda</t>
+          <t>Giralda</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1676,15 +1772,19 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Pinza Aguda" çağrısı</t>
+          <t>"Resurrección: Giralda" çağrısı</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Findorr_Calius</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>Dordoni_Alessandro_Del_Socaccio</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>animede yok</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1693,17 +1793,17 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne_Mosqueda</t>
+          <t>Emilou_Apacci</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne Mosqueda</t>
+          <t>Emilou Apacci</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Dragra</t>
+          <t>Cierva</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1713,12 +1813,12 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Dragra" çağrısı</t>
+          <t>"Resurrección: Cierva" çağrısı</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne_Mosqueda</t>
+          <t>Emilou_Apacci</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -1730,17 +1830,17 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow_Jaegerjaquez</t>
+          <t>Findorr_Calius</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow Jaegerjaquez</t>
+          <t>Findorr Calius</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Pantera</t>
+          <t>Pinza Aguda</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1750,15 +1850,19 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Pantera" çağrısı</t>
+          <t>"Resurrección: Pinza Aguda" çağrısı</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow_Jaegerjaquez</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>Findorr_Calius</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -1767,17 +1871,17 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Luppi_Antenor</t>
+          <t>Franceska_Mila_Rose</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Luppi Antenor</t>
+          <t>Franceska Mila Rose</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Trepadora</t>
+          <t>Leona</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1787,12 +1891,12 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Trepadora" çağrısı</t>
+          <t>"Resurrección: Leona" çağrısı</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Luppi_Antenor</t>
+          <t>Franceska_Mila_Rose</t>
         </is>
       </c>
       <c r="G30" t="inlineStr"/>
@@ -1804,17 +1908,17 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Nelliel_Tu_Odelschwanck</t>
+          <t>Gantenbainne_Mosqueda</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Nelliel Tu Odelschwanck</t>
+          <t>Gantenbainne Mosqueda</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Gamuza</t>
+          <t>Dragra</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1824,12 +1928,12 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Gamuza" çağrısı</t>
+          <t>"Resurrección: Dragra" çağrısı</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Nelliel_Tu_Odelschwanck</t>
+          <t>Gantenbainne_Mosqueda</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -1841,17 +1945,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra_Gilga</t>
+          <t>Ggio_Vega</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra Gilga</t>
+          <t>Ggio Vega</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Santa Teresa</t>
+          <t>Tigre Estoque</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1861,12 +1965,12 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Santa Teresa" çağrısı</t>
+          <t>"Resurrección: Tigre Estoque" çağrısı</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra_Gilga</t>
+          <t>Ggio_Vega</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1878,17 +1982,17 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro_Granz</t>
+          <t>Grimmjow_Jaegerjaquez</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro Granz</t>
+          <t>Grimmjow Jaegerjaquez</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Fornicarás</t>
+          <t>Pantera</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1898,15 +2002,19 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Fornicarás" çağrısı</t>
+          <t>"Resurrección: Pantera" çağrısı</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro_Granz</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>Grimmjow_Jaegerjaquez</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -1915,17 +2023,17 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Tier_Harribel</t>
+          <t>Luppi_Antenor</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Tier Harribel</t>
+          <t>Luppi Antenor</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Tiburón</t>
+          <t>Trepadora</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1935,12 +2043,12 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Tiburón" çağrısı</t>
+          <t>"Resurrección: Trepadora" çağrısı</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Tier_Harribel</t>
+          <t>Luppi_Antenor</t>
         </is>
       </c>
       <c r="G34" t="inlineStr"/>
@@ -1952,17 +2060,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra_Cifer</t>
+          <t>Nelliel_Tu_Odelschwanck</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra Cifer</t>
+          <t>Nelliel Tu Odelschwanck</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Murciélago</t>
+          <t>Gamuza</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1972,12 +2080,12 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Murciélago" çağrısı</t>
+          <t>"Resurrección: Gamuza" çağrısı</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra_Cifer</t>
+          <t>Nelliel_Tu_Odelschwanck</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -1989,17 +2097,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss_Margela</t>
+          <t>Nnoitra_Gilga</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss Margela</t>
+          <t>Nnoitra Gilga</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Extinguir</t>
+          <t>Santa Teresa</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2009,15 +2117,19 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Extinguir" çağrısı</t>
+          <t>"Resurrección: Santa Teresa" çağrısı</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss_Margela</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>Nnoitra_Gilga</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -2026,17 +2138,17 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Yammy_Llargo</t>
+          <t>Szayelaporro_Granz</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Yammy Llargo</t>
+          <t>Szayelaporro Granz</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Ira</t>
+          <t>Fornicarás</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2046,15 +2158,19 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Ira" çağrısı</t>
+          <t>"Resurrección: Fornicarás" çağrısı</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Yammy_Llargo</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>Szayelaporro_Granz</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr"/>
@@ -2063,17 +2179,17 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Zommari_Rureaux</t>
+          <t>Tier_Harribel</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Zommari Rureaux</t>
+          <t>Tier Harribel</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Brujería</t>
+          <t>Tiburón</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2083,15 +2199,19 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Brujería" çağrısı</t>
+          <t>"Resurrección: Tiburón" çağrısı</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Zommari_Rureaux</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>Tier_Harribel</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr"/>
@@ -2100,35 +2220,39 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō_Yamada</t>
+          <t>Ulquiorra_Cifer</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō Yamada</t>
+          <t>Ulquiorra Cifer</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Hisagomaru</t>
+          <t>Murciélago</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>Shikai</t>
+          <t>Resurrección</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Hisagomaru" çağrısı</t>
+          <t>"Resurrección: Murciélago" çağrısı</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō_Yamada</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>Ulquiorra_Cifer</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -2137,32 +2261,32 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Hisagi_Shūhei</t>
+          <t>Wonderweiss_Margela</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Shūhei Hisagi</t>
+          <t>Wonderweiss Margela</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Kazeshini</t>
+          <t>Extinguir</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Shikai</t>
+          <t>Resurrección</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Kazeshini" çağrısı</t>
+          <t>"Resurrección: Extinguir" çağrısı</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Hisagi_Shūhei</t>
+          <t>Wonderweiss_Margela</t>
         </is>
       </c>
       <c r="G40" t="inlineStr"/>
@@ -2174,35 +2298,39 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Ichibē_Hyōsube</t>
+          <t>Yammy_Llargo</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Ichibē Hyōsube</t>
+          <t>Yammy Llargo</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Ichimonji</t>
+          <t>Ira</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>Shikai</t>
+          <t>Resurrección</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Ichimonji" çağrısı</t>
+          <t>"Resurrección: Ira" çağrısı</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Ichibē_Hyōsube</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>Yammy_Llargo</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -2211,35 +2339,39 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Isane_Kotetsu</t>
+          <t>Zommari_Rureaux</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Isane Kotetsu</t>
+          <t>Zommari Rureaux</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Itegumo</t>
+          <t>Brujería</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>Shikai</t>
+          <t>Resurrección</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Itegumo" çağrısı</t>
+          <t>"Resurrección: Brujería" çağrısı</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Isane_Kotetsu</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>Zommari_Rureaux</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr"/>
@@ -2248,17 +2380,17 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Isshin_Kurosaki</t>
+          <t>Hanatarō_Yamada</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Isshin Kurosaki</t>
+          <t>Hanatarō Yamada</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Engetsu</t>
+          <t>Hisagomaru</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -2268,12 +2400,12 @@
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Engetsu" çağrısı</t>
+          <t>"Shikai: Hisagomaru" çağrısı</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Isshin_Kurosaki</t>
+          <t>Hanatarō_Yamada</t>
         </is>
       </c>
       <c r="G43" t="inlineStr"/>
@@ -2285,17 +2417,17 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Izuru_Kira</t>
+          <t>Hisagi_Shūhei</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Izuru Kira</t>
+          <t>Shūhei Hisagi</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Wabisuke</t>
+          <t>Kazeshini</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2305,12 +2437,12 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Wabisuke" çağrısı</t>
+          <t>"Shikai: Kazeshini" çağrısı</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Izuru_Kira</t>
+          <t>Hisagi_Shūhei</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2322,17 +2454,17 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Jūshirō_Ukitake</t>
+          <t>Hiyori_Sarugaki</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Jūshirō Ukitake</t>
+          <t>Hiyori Sarugaki</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Sōgyo no Kotowari</t>
+          <t>Kubikiri Orochi</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2342,12 +2474,12 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Sōgyo no Kotowari" çağrısı</t>
+          <t>"Shikai: Kubikiri Orochi" çağrısı</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Jūshirō_Ukitake</t>
+          <t>Hiyori_Sarugaki</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2359,17 +2491,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Kaien_Shiba</t>
+          <t>Ichibē_Hyōsube</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Kaien Shiba</t>
+          <t>Ichibē Hyōsube</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Nejibana</t>
+          <t>Ichimonji</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -2379,12 +2511,12 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Nejibana" çağrısı</t>
+          <t>"Shikai: Ichimonji" çağrısı</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Kaien_Shiba</t>
+          <t>Ichibē_Hyōsube</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>
@@ -2396,17 +2528,17 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Kenpachi_Zaraki</t>
+          <t>Isane_Kotetsu</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Kenpachi Zaraki</t>
+          <t>Isane Kotetsu</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>Nozarashi</t>
+          <t>Itegumo</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -2416,12 +2548,12 @@
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Nozarashi" çağrısı</t>
+          <t>"Shikai: Itegumo" çağrısı</t>
         </is>
       </c>
       <c r="F47" s="4" t="inlineStr">
         <is>
-          <t>Kenpachi_Zaraki</t>
+          <t>Isane_Kotetsu</t>
         </is>
       </c>
       <c r="G47" t="inlineStr"/>
@@ -2433,17 +2565,17 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>Lisa_Yadōmaru</t>
+          <t>Isshin_Kurosaki</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Lisa Yadōmaru</t>
+          <t>Isshin Kurosaki</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Haguro Tonbo</t>
+          <t>Engetsu</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2453,12 +2585,12 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Haguro Tonbo" çağrısı</t>
+          <t>"Shikai: Engetsu" çağrısı</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>Lisa_Yadōmaru</t>
+          <t>Isshin_Kurosaki</t>
         </is>
       </c>
       <c r="G48" t="inlineStr"/>
@@ -2470,17 +2602,17 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Love_Aikawa</t>
+          <t>Izuru_Kira</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Love Aikawa</t>
+          <t>Izuru Kira</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Tengumaru</t>
+          <t>Wabisuke</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -2490,12 +2622,12 @@
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Tengumaru" çağrısı</t>
+          <t>"Shikai: Wabisuke" çağrısı</t>
         </is>
       </c>
       <c r="F49" s="4" t="inlineStr">
         <is>
-          <t>Love_Aikawa</t>
+          <t>Izuru_Kira</t>
         </is>
       </c>
       <c r="G49" t="inlineStr"/>
@@ -2507,17 +2639,17 @@
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Marechiyo_Ōmaeda</t>
+          <t>Jūshirō_Ukitake</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Marechiyo Ōmaeda</t>
+          <t>Jūshirō Ukitake</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Gegetsuburi</t>
+          <t>Sōgyo no Kotowari</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -2527,12 +2659,12 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Gegetsuburi" çağrısı</t>
+          <t>"Shikai: Sōgyo no Kotowari" çağrısı</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>Marechiyo_Ōmaeda</t>
+          <t>Jūshirō_Ukitake</t>
         </is>
       </c>
       <c r="G50" t="inlineStr"/>
@@ -2544,17 +2676,17 @@
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Momo_Hinamori</t>
+          <t>Kaien_Shiba</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Momo Hinamori</t>
+          <t>Kaien Shiba</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>Tobiume</t>
+          <t>Nejibana</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -2564,12 +2696,12 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Tobiume" çağrısı</t>
+          <t>"Shikai: Nejibana" çağrısı</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
         <is>
-          <t>Momo_Hinamori</t>
+          <t>Kaien_Shiba</t>
         </is>
       </c>
       <c r="G51" t="inlineStr"/>
@@ -2581,17 +2713,17 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>Rangiku_Matsumoto</t>
+          <t>Kenpachi_Zaraki</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Rangiku Matsumoto</t>
+          <t>Kenpachi Zaraki</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Haineko</t>
+          <t>Nozarashi</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -2601,12 +2733,12 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Haineko" çağrısı</t>
+          <t>"Shikai: Nozarashi" çağrısı</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>Rangiku_Matsumoto</t>
+          <t>Kenpachi_Zaraki</t>
         </is>
       </c>
       <c r="G52" t="inlineStr"/>
@@ -2618,17 +2750,17 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Sōsuke_Aizen</t>
+          <t>Lisa_Yadōmaru</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Sōsuke Aizen</t>
+          <t>Lisa Yadōmaru</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Kyōka Suigetsu</t>
+          <t>Haguro Tonbo</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -2638,12 +2770,12 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Kyōka Suigetsu" çağrısı</t>
+          <t>"Shikai: Haguro Tonbo" çağrısı</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
         <is>
-          <t>Sōsuke_Aizen</t>
+          <t>Lisa_Yadōmaru</t>
         </is>
       </c>
       <c r="G53" t="inlineStr"/>
@@ -2655,17 +2787,17 @@
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>Tenjirō_Kirinji</t>
+          <t>Love_Aikawa</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Tenjirō Kirinji</t>
+          <t>Love Aikawa</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>Kinpika</t>
+          <t>Tengumaru</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -2675,12 +2807,12 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Kinpika" çağrısı</t>
+          <t>"Shikai: Tengumaru" çağrısı</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>Tenjirō_Kirinji</t>
+          <t>Love_Aikawa</t>
         </is>
       </c>
       <c r="G54" t="inlineStr"/>
@@ -2692,17 +2824,17 @@
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Yachiru_Kusajishi</t>
+          <t>Marechiyo_Ōmaeda</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Yachiru Kusajishi</t>
+          <t>Marechiyo Ōmaeda</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>Sanpo Kenjū</t>
+          <t>Gegetsuburi</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -2712,12 +2844,12 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Sanpo Kenjū" çağrısı</t>
+          <t>"Shikai: Gegetsuburi" çağrısı</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
         <is>
-          <t>Yachiru_Kusajishi</t>
+          <t>Marechiyo_Ōmaeda</t>
         </is>
       </c>
       <c r="G55" t="inlineStr"/>
@@ -2729,17 +2861,17 @@
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>Yumichika_Ayasegawa</t>
+          <t>Momo_Hinamori</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Yumichika Ayasegawa</t>
+          <t>Momo Hinamori</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Ruri'iro Kujaku</t>
+          <t>Tobiume</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -2749,12 +2881,12 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Ruri'iro Kujaku" çağrısı</t>
+          <t>"Shikai: Tobiume" çağrısı</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Yumichika_Ayasegawa</t>
+          <t>Momo_Hinamori</t>
         </is>
       </c>
       <c r="G56" t="inlineStr"/>
@@ -2763,8 +2895,193 @@
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Rangiku_Matsumoto</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Rangiku Matsumoto</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Haineko</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Shikai</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>"Shikai: Haineko" çağrısı</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Rangiku_Matsumoto</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr"/>
+    </row>
     <row r="58">
-      <c r="A58" s="5" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Sōsuke_Aizen</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Sōsuke Aizen</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Kyōka Suigetsu</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Shikai</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>"Shikai: Kyōka Suigetsu" çağrısı</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Sōsuke_Aizen</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Tenjirō_Kirinji</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Tenjirō Kirinji</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Kinpika</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Shikai</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>"Shikai: Kinpika" çağrısı</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Tenjirō_Kirinji</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Yachiru_Kusajishi</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Yachiru Kusajishi</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Sanpo Kenjū</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Shikai</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>"Shikai: Sanpo Kenjū" çağrısı</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Yachiru_Kusajishi</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Yumichika_Ayasegawa</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Yumichika Ayasegawa</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Ruri'iro Kujaku</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Shikai</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>"Shikai: Ruri'iro Kujaku" çağrısı</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Yumichika_Ayasegawa</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>Dosyayı audio_in/bankai/ altına, dosya_adı sütunundaki adla bırak. Uzantı farketmez.</t>
         </is>
@@ -2772,7 +3089,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"aranıyor,bulundu,animede yok,belirsiz"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Ichibē'nin Bankai'si Shinuchi alanında; ses dosyası notları korunur
- Wiki Ichibē'nin Bankai'sini "shinuchi" alanında tutuyor; kazıyıcı
  okumadığı için havuzda Shikai'si (Ichimonji) duruyordu. Artık
  "Shirafude Ichimonji" (Bankai). Bu alan yalnız onda var.
- make_audio_sheet: id'si veriyle eşleşmeyen satırları (alta yazılmış
  notlar, listeden çıkan karakterler) siliyordu; Ozgur'un Bankai
  sayfasının altındaki not böyle kayboldu. Artık bu satırlar sayfanın
  altına aynen taşınıyor ve eski dosya her seferinde audio_in/yedek/
  altına kopyalanıyor.
- Çalışma dosyasında Ichibē: bulundu (Ozgur'un notu).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bleachdle-ses.xlsx
+++ b/bleachdle-ses.xlsx
@@ -895,17 +895,17 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Ichigo_Kurosaki</t>
+          <t>Ichibē_Hyōsube</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Ichigo Kurosaki</t>
+          <t>Ichibē Hyōsube</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Tensa Zangetsu</t>
+          <t>Shirafude Ichimonji</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -915,12 +915,12 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Tensa Zangetsu" çağrısı</t>
+          <t>"Bankai: Shirafude Ichimonji" çağrısı</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Ichigo_Kurosaki</t>
+          <t>Ichibē_Hyōsube</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -931,22 +931,26 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Shinuchi (Ichibē'nin Bankai karşılığı); klip Ozgur'un notuyla eklendi</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Ikkaku_Madarame</t>
+          <t>Ichigo_Kurosaki</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Ikkaku Madarame</t>
+          <t>Ichigo Kurosaki</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Ryūmon Hōzukimaru</t>
+          <t>Tensa Zangetsu</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -956,12 +960,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Ryūmon Hōzukimaru" çağrısı</t>
+          <t>"Bankai: Tensa Zangetsu" çağrısı</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Ikkaku_Madarame</t>
+          <t>Ichigo_Kurosaki</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -977,17 +981,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Kaname_Tōsen</t>
+          <t>Ikkaku_Madarame</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Kaname Tōsen</t>
+          <t>Ikkaku Madarame</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Suzumushi Tsuishiki: Enma Kōrogi</t>
+          <t>Ryūmon Hōzukimaru</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -997,12 +1001,12 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Suzumushi Tsuishiki: Enma Kōrogi" çağrısı</t>
+          <t>"Bankai: Ryūmon Hōzukimaru" çağrısı</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Kaname_Tōsen</t>
+          <t>Ikkaku_Madarame</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1018,17 +1022,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Kensei_Muguruma</t>
+          <t>Kaname_Tōsen</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Kensei Muguruma</t>
+          <t>Kaname Tōsen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tekken Tachikaze</t>
+          <t>Suzumushi Tsuishiki: Enma Kōrogi</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1038,12 +1042,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Tekken Tachikaze" çağrısı</t>
+          <t>"Bankai: Suzumushi Tsuishiki: Enma Kōrogi" çağrısı</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Kensei_Muguruma</t>
+          <t>Kaname_Tōsen</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1059,17 +1063,17 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Kisuke_Urahara</t>
+          <t>Kensei_Muguruma</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Kisuke Urahara</t>
+          <t>Kensei Muguruma</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Kannonbiraki Benihime Aratame</t>
+          <t>Tekken Tachikaze</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1079,12 +1083,12 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Kannonbiraki Benihime Aratame" çağrısı</t>
+          <t>"Bankai: Tekken Tachikaze" çağrısı</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Kisuke_Urahara</t>
+          <t>Kensei_Muguruma</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1100,17 +1104,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Mayuri_Kurotsuchi</t>
+          <t>Kisuke_Urahara</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Mayuri Kurotsuchi</t>
+          <t>Kisuke Urahara</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Konjiki Ashisogi Jizō</t>
+          <t>Kannonbiraki Benihime Aratame</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1120,12 +1124,12 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Konjiki Ashisogi Jizō" çağrısı</t>
+          <t>"Bankai: Kannonbiraki Benihime Aratame" çağrısı</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Mayuri_Kurotsuchi</t>
+          <t>Kisuke_Urahara</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1141,17 +1145,17 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Renji_Abarai</t>
+          <t>Mayuri_Kurotsuchi</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Renji Abarai</t>
+          <t>Mayuri Kurotsuchi</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Sōō Zabimaru</t>
+          <t>Konjiki Ashisogi Jizō</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1161,12 +1165,12 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Sōō Zabimaru" çağrısı</t>
+          <t>"Bankai: Konjiki Ashisogi Jizō" çağrısı</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Renji_Abarai</t>
+          <t>Mayuri_Kurotsuchi</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1182,17 +1186,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Retsu_Unohana</t>
+          <t>Renji_Abarai</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Retsu Unohana</t>
+          <t>Renji Abarai</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Minazuki</t>
+          <t>Sōō Zabimaru</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1202,12 +1206,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Minazuki" çağrısı</t>
+          <t>"Bankai: Sōō Zabimaru" çağrısı</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Retsu_Unohana</t>
+          <t>Renji_Abarai</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1223,17 +1227,17 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Rukia_Kuchiki</t>
+          <t>Retsu_Unohana</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Rukia Kuchiki</t>
+          <t>Retsu Unohana</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Hakka no Togame</t>
+          <t>Minazuki</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1243,12 +1247,12 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Hakka no Togame" çağrısı</t>
+          <t>"Bankai: Minazuki" çağrısı</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Rukia_Kuchiki</t>
+          <t>Retsu_Unohana</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1264,17 +1268,17 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Rōjūrō_Ōtoribashi</t>
+          <t>Rukia_Kuchiki</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Rōjūrō Ōtoribashi</t>
+          <t>Rukia Kuchiki</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Kinshara Butōdan</t>
+          <t>Hakka no Togame</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1284,12 +1288,12 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Kinshara Butōdan" çağrısı</t>
+          <t>"Bankai: Hakka no Togame" çağrısı</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Rōjūrō_Ōtoribashi</t>
+          <t>Rukia_Kuchiki</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1305,17 +1309,17 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Sajin_Komamura</t>
+          <t>Rōjūrō_Ōtoribashi</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sajin Komamura</t>
+          <t>Rōjūrō Ōtoribashi</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Kokujō Tengen Myō'ō</t>
+          <t>Kinshara Butōdan</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1325,12 +1329,12 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Kokujō Tengen Myō'ō" çağrısı</t>
+          <t>"Bankai: Kinshara Butōdan" çağrısı</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Sajin_Komamura</t>
+          <t>Rōjūrō_Ōtoribashi</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1346,17 +1350,17 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Senjumaru_Shutara</t>
+          <t>Sajin_Komamura</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Senjumaru Shutara</t>
+          <t>Sajin Komamura</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Shatatsu Karagara Shigarami no Tsuji</t>
+          <t>Kokujō Tengen Myō'ō</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1366,12 +1370,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Shatatsu Karagara Shigarami no Tsuji" çağrısı</t>
+          <t>"Bankai: Kokujō Tengen Myō'ō" çağrısı</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Senjumaru_Shutara</t>
+          <t>Sajin_Komamura</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1387,17 +1391,17 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Shinji_Hirako</t>
+          <t>Senjumaru_Shutara</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Shinji Hirako</t>
+          <t>Senjumaru Shutara</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Sakashima Yokoshima Happōfusagari</t>
+          <t>Shatatsu Karagara Shigarami no Tsuji</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1407,12 +1411,12 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Sakashima Yokoshima Happōfusagari" çağrısı</t>
+          <t>"Bankai: Shatatsu Karagara Shigarami no Tsuji" çağrısı</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Shinji_Hirako</t>
+          <t>Senjumaru_Shutara</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1428,17 +1432,17 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Shunsui_Kyōraku</t>
+          <t>Shinji_Hirako</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Shunsui Kyōraku</t>
+          <t>Shinji Hirako</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Katen Kyōkotsu: Karamatsu Shinjū</t>
+          <t>Sakashima Yokoshima Happōfusagari</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1448,12 +1452,12 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Katen Kyōkotsu: Karamatsu Shinjū" çağrısı</t>
+          <t>"Bankai: Sakashima Yokoshima Happōfusagari" çağrısı</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Shunsui_Kyōraku</t>
+          <t>Shinji_Hirako</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1469,17 +1473,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Sui_Feng</t>
+          <t>Shunsui_Kyōraku</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Sui-Feng</t>
+          <t>Shunsui Kyōraku</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Jakuhō Raikōben</t>
+          <t>Katen Kyōkotsu: Karamatsu Shinjū</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1489,12 +1493,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Jakuhō Raikōben" çağrısı</t>
+          <t>"Bankai: Katen Kyōkotsu: Karamatsu Shinjū" çağrısı</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Sui_Feng</t>
+          <t>Shunsui_Kyōraku</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1510,17 +1514,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Tōshirō_Hitsugaya</t>
+          <t>Sui_Feng</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Tōshirō Hitsugaya</t>
+          <t>Sui-Feng</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Daiguren Hyōrinmaru</t>
+          <t>Jakuhō Raikōben</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1530,12 +1534,12 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>"Bankai: Daiguren Hyōrinmaru" çağrısı</t>
+          <t>"Bankai: Jakuhō Raikōben" çağrısı</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Tōshirō_Hitsugaya</t>
+          <t>Sui_Feng</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1551,32 +1555,32 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Aaroniero_Arruruerie</t>
+          <t>Tōshirō_Hitsugaya</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Aaroniero Arruruerie</t>
+          <t>Tōshirō Hitsugaya</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Glotonería</t>
+          <t>Daiguren Hyōrinmaru</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Resurrección</t>
+          <t>Bankai</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Glotonería" çağrısı</t>
+          <t>"Bankai: Daiguren Hyōrinmaru" çağrısı</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Aaroniero_Arruruerie</t>
+          <t>Tōshirō_Hitsugaya</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1592,17 +1596,17 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Baraggan_Louisenbairn</t>
+          <t>Aaroniero_Arruruerie</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Baraggan Louisenbairn</t>
+          <t>Aaroniero Arruruerie</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Arrogante</t>
+          <t>Glotonería</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1612,12 +1616,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Arrogante" çağrısı</t>
+          <t>"Resurrección: Glotonería" çağrısı</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Baraggan_Louisenbairn</t>
+          <t>Aaroniero_Arruruerie</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1633,17 +1637,17 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Cirucci_Sanderwicci</t>
+          <t>Baraggan_Louisenbairn</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Cirucci Sanderwicci</t>
+          <t>Baraggan Louisenbairn</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Golondrina</t>
+          <t>Arrogante</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1653,12 +1657,12 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Golondrina" çağrısı</t>
+          <t>"Resurrección: Arrogante" çağrısı</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Cirucci_Sanderwicci</t>
+          <t>Baraggan_Louisenbairn</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1674,17 +1678,17 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Coyote_Starrk</t>
+          <t>Cirucci_Sanderwicci</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Coyote Starrk</t>
+          <t>Cirucci Sanderwicci</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Los Lobos</t>
+          <t>Golondrina</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1694,12 +1698,12 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Los Lobos" çağrısı</t>
+          <t>"Resurrección: Golondrina" çağrısı</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Coyote_Starrk</t>
+          <t>Cirucci_Sanderwicci</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1715,17 +1719,17 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Cyan_Sung_Sun</t>
+          <t>Coyote_Starrk</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Cyan Sung-Sun</t>
+          <t>Coyote Starrk</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Anaconda</t>
+          <t>Los Lobos</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1735,15 +1739,19 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Anaconda" çağrısı</t>
+          <t>"Resurrección: Los Lobos" çağrısı</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Cyan_Sung_Sun</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>Coyote_Starrk</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1752,17 +1760,17 @@
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Dordoni_Alessandro_Del_Socaccio</t>
+          <t>Cyan_Sung_Sun</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Dordoni Alessandro Del Socaccio</t>
+          <t>Cyan Sung-Sun</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Giralda</t>
+          <t>Anaconda</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1772,19 +1780,15 @@
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Giralda" çağrısı</t>
+          <t>"Resurrección: Anaconda" çağrısı</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Dordoni_Alessandro_Del_Socaccio</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>animede yok</t>
-        </is>
-      </c>
+          <t>Cyan_Sung_Sun</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1793,17 +1797,17 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Emilou_Apacci</t>
+          <t>Dordoni_Alessandro_Del_Socaccio</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Emilou Apacci</t>
+          <t>Dordoni Alessandro Del Socaccio</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Cierva</t>
+          <t>Giralda</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1813,15 +1817,19 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Cierva" çağrısı</t>
+          <t>"Resurrección: Giralda" çağrısı</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Emilou_Apacci</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>Dordoni_Alessandro_Del_Socaccio</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>animede yok</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr"/>
@@ -1830,17 +1838,17 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Findorr_Calius</t>
+          <t>Emilou_Apacci</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Findorr Calius</t>
+          <t>Emilou Apacci</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Pinza Aguda</t>
+          <t>Cierva</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1850,19 +1858,15 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Pinza Aguda" çağrısı</t>
+          <t>"Resurrección: Cierva" çağrısı</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>Findorr_Calius</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>bulundu</t>
-        </is>
-      </c>
+          <t>Emilou_Apacci</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
@@ -1871,17 +1875,17 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Franceska_Mila_Rose</t>
+          <t>Findorr_Calius</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Franceska Mila Rose</t>
+          <t>Findorr Calius</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Leona</t>
+          <t>Pinza Aguda</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1891,15 +1895,19 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Leona" çağrısı</t>
+          <t>"Resurrección: Pinza Aguda" çağrısı</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Franceska_Mila_Rose</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>Findorr_Calius</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr"/>
@@ -1908,17 +1916,17 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne_Mosqueda</t>
+          <t>Franceska_Mila_Rose</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne Mosqueda</t>
+          <t>Franceska Mila Rose</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Dragra</t>
+          <t>Leona</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1928,12 +1936,12 @@
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Dragra" çağrısı</t>
+          <t>"Resurrección: Leona" çağrısı</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Gantenbainne_Mosqueda</t>
+          <t>Franceska_Mila_Rose</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -1945,17 +1953,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Ggio_Vega</t>
+          <t>Gantenbainne_Mosqueda</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Ggio Vega</t>
+          <t>Gantenbainne Mosqueda</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Tigre Estoque</t>
+          <t>Dragra</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1965,12 +1973,12 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Tigre Estoque" çağrısı</t>
+          <t>"Resurrección: Dragra" çağrısı</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Ggio_Vega</t>
+          <t>Gantenbainne_Mosqueda</t>
         </is>
       </c>
       <c r="G32" t="inlineStr"/>
@@ -1982,17 +1990,17 @@
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow_Jaegerjaquez</t>
+          <t>Ggio_Vega</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow Jaegerjaquez</t>
+          <t>Ggio Vega</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Pantera</t>
+          <t>Tigre Estoque</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -2002,19 +2010,15 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Pantera" çağrısı</t>
+          <t>"Resurrección: Tigre Estoque" çağrısı</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Grimmjow_Jaegerjaquez</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>bulundu</t>
-        </is>
-      </c>
+          <t>Ggio_Vega</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -2023,17 +2027,17 @@
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Luppi_Antenor</t>
+          <t>Grimmjow_Jaegerjaquez</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Luppi Antenor</t>
+          <t>Grimmjow Jaegerjaquez</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Trepadora</t>
+          <t>Pantera</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -2043,15 +2047,19 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Trepadora" çağrısı</t>
+          <t>"Resurrección: Pantera" çağrısı</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>Luppi_Antenor</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>Grimmjow_Jaegerjaquez</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr"/>
@@ -2060,17 +2068,17 @@
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Nelliel_Tu_Odelschwanck</t>
+          <t>Luppi_Antenor</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Nelliel Tu Odelschwanck</t>
+          <t>Luppi Antenor</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Gamuza</t>
+          <t>Trepadora</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -2080,12 +2088,12 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Gamuza" çağrısı</t>
+          <t>"Resurrección: Trepadora" çağrısı</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Nelliel_Tu_Odelschwanck</t>
+          <t>Luppi_Antenor</t>
         </is>
       </c>
       <c r="G35" t="inlineStr"/>
@@ -2097,17 +2105,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra_Gilga</t>
+          <t>Nelliel_Tu_Odelschwanck</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra Gilga</t>
+          <t>Nelliel Tu Odelschwanck</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Santa Teresa</t>
+          <t>Gamuza</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -2117,19 +2125,15 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Santa Teresa" çağrısı</t>
+          <t>"Resurrección: Gamuza" çağrısı</t>
         </is>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Nnoitra_Gilga</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>bulundu</t>
-        </is>
-      </c>
+          <t>Nelliel_Tu_Odelschwanck</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
@@ -2138,17 +2142,17 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro_Granz</t>
+          <t>Nnoitra_Gilga</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro Granz</t>
+          <t>Nnoitra Gilga</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Fornicarás</t>
+          <t>Santa Teresa</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -2158,12 +2162,12 @@
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Fornicarás" çağrısı</t>
+          <t>"Resurrección: Santa Teresa" çağrısı</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Szayelaporro_Granz</t>
+          <t>Nnoitra_Gilga</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2179,17 +2183,17 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>Tier_Harribel</t>
+          <t>Szayelaporro_Granz</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Tier Harribel</t>
+          <t>Szayelaporro Granz</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Tiburón</t>
+          <t>Fornicarás</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -2199,12 +2203,12 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Tiburón" çağrısı</t>
+          <t>"Resurrección: Fornicarás" çağrısı</t>
         </is>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Tier_Harribel</t>
+          <t>Szayelaporro_Granz</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2220,17 +2224,17 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra_Cifer</t>
+          <t>Tier_Harribel</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra Cifer</t>
+          <t>Tier Harribel</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>Murciélago</t>
+          <t>Tiburón</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -2240,12 +2244,12 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Murciélago" çağrısı</t>
+          <t>"Resurrección: Tiburón" çağrısı</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Ulquiorra_Cifer</t>
+          <t>Tier_Harribel</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2261,17 +2265,17 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss_Margela</t>
+          <t>Ulquiorra_Cifer</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss Margela</t>
+          <t>Ulquiorra Cifer</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Extinguir</t>
+          <t>Murciélago</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -2281,15 +2285,19 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Extinguir" çağrısı</t>
+          <t>"Resurrección: Murciélago" çağrısı</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>Wonderweiss_Margela</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>Ulquiorra_Cifer</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr"/>
@@ -2298,17 +2306,17 @@
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Yammy_Llargo</t>
+          <t>Wonderweiss_Margela</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Yammy Llargo</t>
+          <t>Wonderweiss Margela</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>Ira</t>
+          <t>Extinguir</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -2318,19 +2326,15 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Ira" çağrısı</t>
+          <t>"Resurrección: Extinguir" çağrısı</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Yammy_Llargo</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>bulundu</t>
-        </is>
-      </c>
+          <t>Wonderweiss_Margela</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
@@ -2339,17 +2343,17 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>Zommari_Rureaux</t>
+          <t>Yammy_Llargo</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Zommari Rureaux</t>
+          <t>Yammy Llargo</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Brujería</t>
+          <t>Ira</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -2359,12 +2363,12 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>"Resurrección: Brujería" çağrısı</t>
+          <t>"Resurrección: Ira" çağrısı</t>
         </is>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>Zommari_Rureaux</t>
+          <t>Yammy_Llargo</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2380,35 +2384,39 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō_Yamada</t>
+          <t>Zommari_Rureaux</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō Yamada</t>
+          <t>Zommari Rureaux</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>Hisagomaru</t>
+          <t>Brujería</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>Shikai</t>
+          <t>Resurrección</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Hisagomaru" çağrısı</t>
+          <t>"Resurrección: Brujería" çağrısı</t>
         </is>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Hanatarō_Yamada</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>Zommari_Rureaux</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>bulundu</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr"/>
@@ -2417,17 +2425,17 @@
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>Hisagi_Shūhei</t>
+          <t>Hanatarō_Yamada</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Shūhei Hisagi</t>
+          <t>Hanatarō Yamada</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Kazeshini</t>
+          <t>Hisagomaru</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2437,12 +2445,12 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Kazeshini" çağrısı</t>
+          <t>"Shikai: Hisagomaru" çağrısı</t>
         </is>
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>Hisagi_Shūhei</t>
+          <t>Hanatarō_Yamada</t>
         </is>
       </c>
       <c r="G44" t="inlineStr"/>
@@ -2454,17 +2462,17 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Hiyori_Sarugaki</t>
+          <t>Hisagi_Shūhei</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Hiyori Sarugaki</t>
+          <t>Shūhei Hisagi</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>Kubikiri Orochi</t>
+          <t>Kazeshini</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -2474,12 +2482,12 @@
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Kubikiri Orochi" çağrısı</t>
+          <t>"Shikai: Kazeshini" çağrısı</t>
         </is>
       </c>
       <c r="F45" s="4" t="inlineStr">
         <is>
-          <t>Hiyori_Sarugaki</t>
+          <t>Hisagi_Shūhei</t>
         </is>
       </c>
       <c r="G45" t="inlineStr"/>
@@ -2491,17 +2499,17 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Ichibē_Hyōsube</t>
+          <t>Hiyori_Sarugaki</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Ichibē Hyōsube</t>
+          <t>Hiyori Sarugaki</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Ichimonji</t>
+          <t>Kubikiri Orochi</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -2511,12 +2519,12 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>"Shikai: Ichimonji" çağrısı</t>
+          <t>"Shikai: Kubikiri Orochi" çağrısı</t>
         </is>
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>Ichibē_Hyōsube</t>
+          <t>Hiyori_Sarugaki</t>
         </is>
       </c>
       <c r="G46" t="inlineStr"/>

</xml_diff>